<commit_message>
Eliminación de direccion, telefono, mail, y coordenadas en la tabla de entidades, ya que ahora se recogen en sus sedes físicas
</commit_message>
<xml_diff>
--- a/Datos.xlsx
+++ b/Datos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EAPN\eapn_mapa_servicios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD2EB94C-9E6A-4E39-83CC-B2B1CE4473BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1686764A-F866-4909-9E23-6028EC13311D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{87297B91-5DF4-4B0C-8369-AA06C1FF636B}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="DatosExternos_1" localSheetId="0" hidden="1">Entidades!$A$1:$I$45</definedName>
-    <definedName name="DatosExternos_1" localSheetId="1" hidden="1">Sedes!$A$1:$I$31</definedName>
+    <definedName name="DatosExternos_1" localSheetId="1" hidden="1">Sedes!$A$1:$I$66</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="734" uniqueCount="538">
   <si>
     <t>entidad_id</t>
   </si>
@@ -804,439 +804,869 @@
     <t>Palencia</t>
   </si>
   <si>
-    <t>C. del Puente, 30, 05600 El Barco de Ávila, Ávila</t>
-  </si>
-  <si>
-    <t>El Barco de Ávila</t>
-  </si>
-  <si>
     <t>Ávila</t>
   </si>
   <si>
-    <t>05600</t>
-  </si>
-  <si>
-    <t>C/ Manuel Altolaguirre, s/n. 09006. Burgos.</t>
-  </si>
-  <si>
     <t>09006</t>
   </si>
   <si>
-    <t>C/Padre Aramburu, 2 09006 Burgos</t>
-  </si>
-  <si>
-    <t>Avda/Castilla y León, 34 09006 Burgos</t>
-  </si>
-  <si>
-    <t>Avenida Castilla y León 22, 2ªPlanta. 09006, Burgos CC Camino de la plata</t>
-  </si>
-  <si>
-    <t>Calle Martínez Salazar, 8, 24700 Astorga</t>
-  </si>
-  <si>
-    <t>Astorga</t>
-  </si>
-  <si>
-    <t>Calle Real, 63, 24400 Ponferrada</t>
-  </si>
-  <si>
-    <t>Ponferrada</t>
-  </si>
-  <si>
-    <t>Avenida de La Libertad, 31, 24400 Ponferrada</t>
-  </si>
-  <si>
-    <t>Avenida El Bierzo, 22, 24300 Bembibre</t>
-  </si>
-  <si>
-    <t>Bembibre</t>
-  </si>
-  <si>
-    <t>24700</t>
-  </si>
-  <si>
-    <t>24400</t>
-  </si>
-  <si>
-    <t>24300</t>
-  </si>
-  <si>
-    <t>Calle María Zapata, 21, 24750 La Bañeza</t>
-  </si>
-  <si>
-    <t>24757</t>
-  </si>
-  <si>
-    <t>La Bañeza</t>
-  </si>
-  <si>
-    <t>Calle Valorca, 2, 32300, O Barco de Valdeorras</t>
-  </si>
-  <si>
-    <t>32300</t>
-  </si>
-  <si>
-    <t>O Barco de Valdeorras</t>
-  </si>
-  <si>
-    <t>Calle Lorenzo Miguélez, 2, 24350, Veguellina del Órbigo</t>
-  </si>
-  <si>
-    <t>24350</t>
-  </si>
-  <si>
-    <t>Veguellina del Órbigo</t>
-  </si>
-  <si>
-    <t>Rúa Carreira, 5, 32356, Petín</t>
-  </si>
-  <si>
-    <t>32356</t>
-  </si>
-  <si>
-    <t>Petín</t>
-  </si>
-  <si>
-    <t>Plaza San Nicolás, 3-24420 Fabero</t>
-  </si>
-  <si>
-    <t>24420</t>
-  </si>
-  <si>
-    <t>Fabero</t>
-  </si>
-  <si>
-    <t>web@caritasastorga.com</t>
-  </si>
-  <si>
-    <t>Calle Sierra Pambley, Nº10, Cp: 24286, Hospital de Órbigo, León</t>
-  </si>
-  <si>
-    <t>24286</t>
-  </si>
-  <si>
-    <t>Hospital de Orbigo</t>
-  </si>
-  <si>
-    <t>Calle Sierra Pambley, 6, 24003 León, España</t>
-  </si>
-  <si>
     <t>24003</t>
   </si>
   <si>
-    <t>C/ Campos Góticos s/n 2ª Planta (despachos 18-20)</t>
-  </si>
-  <si>
-    <t>Bajos del Toralín, local 18</t>
-  </si>
-  <si>
-    <t>24005</t>
-  </si>
-  <si>
-    <t>24404</t>
-  </si>
-  <si>
-    <t>Calle Bolívar, 33</t>
-  </si>
-  <si>
-    <t>salamanca@ymca.es</t>
-  </si>
-  <si>
     <t>Salamanca</t>
   </si>
   <si>
     <t>37004</t>
   </si>
   <si>
-    <t>Calle Brocheros, 15</t>
-  </si>
-  <si>
-    <t>Pasaje Marquesina, 15</t>
-  </si>
-  <si>
-    <t>valladolid@ymca.es</t>
-  </si>
-  <si>
     <t>47004</t>
   </si>
   <si>
-    <t>Plaza del Ayuntamiento s/n</t>
-  </si>
-  <si>
-    <t>salduero.ingles@ymca.es</t>
-  </si>
-  <si>
-    <t>42156</t>
-  </si>
-  <si>
-    <t>Salduero</t>
-  </si>
-  <si>
     <t>Soria</t>
   </si>
   <si>
-    <t>C/ Santa Clara, 15 Bajo</t>
-  </si>
-  <si>
-    <t>fsgsalamanca@gitanos.org</t>
-  </si>
-  <si>
-    <t>Avenida Castilla 47</t>
-  </si>
-  <si>
-    <t>susana.corral@gitanos.org</t>
-  </si>
-  <si>
-    <t>Aranda de Duero</t>
-  </si>
-  <si>
-    <t>C/ Averroes, 12. Local</t>
-  </si>
-  <si>
-    <t>fsgburgos@gitanos.org</t>
-  </si>
-  <si>
-    <t>Cardenal Cisneros, 65</t>
-  </si>
-  <si>
-    <t>fsgleon@gitanos.org</t>
-  </si>
-  <si>
-    <t>fsgpalencia@gitanos.org</t>
-  </si>
-  <si>
-    <t>C/ Verbena, 6 Local</t>
-  </si>
-  <si>
-    <t>fsgvalladolid@gitanos.org</t>
-  </si>
-  <si>
-    <t>Av. de Galicia, 10-D</t>
-  </si>
-  <si>
-    <t>fsgzamora@gitanos.org</t>
-  </si>
-  <si>
     <t>Zamora</t>
   </si>
   <si>
-    <t>fsgsegovia@gitanos.org</t>
-  </si>
-  <si>
     <t>Segovia</t>
   </si>
   <si>
-    <t>42.455701664731095, -6.056329247321293</t>
-  </si>
-  <si>
-    <t>42.54755251146814, -6.5986127184827605</t>
-  </si>
-  <si>
-    <t>42.554069930450396, -6.597971016638292</t>
-  </si>
-  <si>
-    <t>42.61719290056674, -6.415971445470651</t>
-  </si>
-  <si>
-    <t>42.30084051487661, -5.904171789030497</t>
-  </si>
-  <si>
-    <t>42.41709954857173, -6.982751482276468</t>
-  </si>
-  <si>
-    <t>42.43461918659991, -5.883491230138437</t>
-  </si>
-  <si>
-    <t>42.38301324440409, -7.125684231984689</t>
-  </si>
-  <si>
-    <t>42.76377710484809, -6.628068303134523</t>
-  </si>
-  <si>
-    <t>42.46227480998277, -5.88191203446407</t>
-  </si>
-  <si>
-    <t>42.59928582539271, -5.568405930131844</t>
-  </si>
-  <si>
-    <t>40.97368790790581, -5.65400940420515</t>
-  </si>
-  <si>
-    <t>40.97407503937069, -5.655142626507726</t>
-  </si>
-  <si>
-    <t>41.64580125974085, -4.724172991527865</t>
-  </si>
-  <si>
-    <t>41.88927533195551, -2.797357887829948</t>
-  </si>
-  <si>
-    <t>40.962331349586854, -5.659591148382658</t>
-  </si>
-  <si>
-    <t>42.35773517716968, -3.673810562664731</t>
-  </si>
-  <si>
-    <t>42.35757804583617, -3.6718304651730724</t>
-  </si>
-  <si>
-    <t>42.6016733273476, -5.591780291489855</t>
-  </si>
-  <si>
-    <t>41.651479836705136, -4.715883943664921</t>
-  </si>
-  <si>
-    <t>C. San Marcos, 7, 34001 Palencia</t>
-  </si>
-  <si>
-    <t>42.0092160611433, -4.535654343650786</t>
-  </si>
-  <si>
-    <t>41.50938069379088, -5.7506633743495374</t>
-  </si>
-  <si>
-    <t>C. Anselmo Carretero, s/n, sección B, 40003 Segovia</t>
-  </si>
-  <si>
-    <t>40.95411944421286, -4.110450233885097</t>
-  </si>
-  <si>
-    <t>42,455701</t>
-  </si>
-  <si>
-    <t>-6,056329</t>
-  </si>
-  <si>
-    <t>42,547552</t>
-  </si>
-  <si>
-    <t>-6,598612</t>
-  </si>
-  <si>
-    <t>42,554069</t>
-  </si>
-  <si>
-    <t>-6,597971</t>
-  </si>
-  <si>
-    <t>42,617192</t>
-  </si>
-  <si>
-    <t>-6,415971</t>
-  </si>
-  <si>
-    <t>42,300840</t>
-  </si>
-  <si>
-    <t>-5,904171</t>
-  </si>
-  <si>
-    <t>42,417099</t>
-  </si>
-  <si>
-    <t>-6,982751</t>
-  </si>
-  <si>
-    <t>42,434619</t>
-  </si>
-  <si>
-    <t>-5,883491</t>
-  </si>
-  <si>
-    <t>42,383013</t>
-  </si>
-  <si>
-    <t>-7,125684</t>
-  </si>
-  <si>
-    <t>42,763777</t>
-  </si>
-  <si>
-    <t>-6,628068</t>
-  </si>
-  <si>
-    <t>42,462274</t>
-  </si>
-  <si>
-    <t>-5,881912</t>
-  </si>
-  <si>
-    <t>42,599285</t>
-  </si>
-  <si>
-    <t>-5,568405</t>
-  </si>
-  <si>
-    <t>40,973687</t>
-  </si>
-  <si>
-    <t>-5,654009</t>
-  </si>
-  <si>
-    <t>40,974075</t>
-  </si>
-  <si>
-    <t>-5,655142</t>
-  </si>
-  <si>
-    <t>41,645801</t>
-  </si>
-  <si>
-    <t>-4,724172</t>
-  </si>
-  <si>
-    <t>41,889275</t>
-  </si>
-  <si>
-    <t>-2,797357</t>
-  </si>
-  <si>
-    <t>40,962331</t>
-  </si>
-  <si>
-    <t>-5,659591</t>
-  </si>
-  <si>
-    <t>42,357735</t>
-  </si>
-  <si>
-    <t>-3,673810</t>
-  </si>
-  <si>
-    <t>42,357578</t>
-  </si>
-  <si>
-    <t>-3,671830</t>
-  </si>
-  <si>
-    <t>42,601673</t>
-  </si>
-  <si>
-    <t>5.,917802</t>
-  </si>
-  <si>
-    <t>42,009216</t>
-  </si>
-  <si>
-    <t>-4,535654</t>
-  </si>
-  <si>
-    <t>41,651479</t>
-  </si>
-  <si>
-    <t>-4,715883</t>
-  </si>
-  <si>
-    <t>41,509380</t>
-  </si>
-  <si>
-    <t>-5,750663</t>
-  </si>
-  <si>
-    <t>40,954119</t>
-  </si>
-  <si>
-    <t>-4,110450</t>
+    <t>Calle Don Sancho, 17, 47002 Valladolid</t>
+  </si>
+  <si>
+    <t>valladolid@accem.es</t>
+  </si>
+  <si>
+    <t>47002</t>
+  </si>
+  <si>
+    <t>Paseo de los Robles, 29, 37004 Salamanca</t>
+  </si>
+  <si>
+    <t>salamanca@accem.es</t>
+  </si>
+  <si>
+    <t>Calle Morillo, 7, 40002 Segovia</t>
+  </si>
+  <si>
+    <t>segovia@accem.es</t>
+  </si>
+  <si>
+    <t>Plaza Bernardo Robles, 9, Soria</t>
+  </si>
+  <si>
+    <t>soria@accem.es</t>
+  </si>
+  <si>
+    <t>Calle Duque de Alba, 6. Local 15., 05001 Ávila</t>
+  </si>
+  <si>
+    <t>Avenida Cantabria 37, bajo, 09006 Burgos</t>
+  </si>
+  <si>
+    <t>burgos@accem.es</t>
+  </si>
+  <si>
+    <t>Calle de la Anunciata, 48, bajo, 24010 Trobajo del Camino, León</t>
+  </si>
+  <si>
+    <t>42002</t>
+  </si>
+  <si>
+    <t>soria</t>
+  </si>
+  <si>
+    <t>05001</t>
+  </si>
+  <si>
+    <t>24010</t>
+  </si>
+  <si>
+    <t>Trobajo del Camino</t>
+  </si>
+  <si>
+    <t>avila@accem.es</t>
+  </si>
+  <si>
+    <t>Calle San Patricio, 5-7, C.P. 37002</t>
+  </si>
+  <si>
+    <t>salamanca@cepaim.org</t>
+  </si>
+  <si>
+    <t>37002</t>
+  </si>
+  <si>
+    <t>Ronda Eloy Sanz Villa 6 bajo, C.P. 42003</t>
+  </si>
+  <si>
+    <t>soria@cepaim.org</t>
+  </si>
+  <si>
+    <t>42003</t>
+  </si>
+  <si>
+    <t>Calle Miguel Íscar 16, Portal 1, 3º, C.P. 47001</t>
+  </si>
+  <si>
+    <t>valladolid@cepaim.org</t>
+  </si>
+  <si>
+    <t>47001</t>
+  </si>
+  <si>
+    <t>C. del Arzobispo José Delicado, 5, 47014 Valladolid, España</t>
+  </si>
+  <si>
+    <t>47014</t>
+  </si>
+  <si>
+    <t>C. Pólvora, 6, 47005 Valladolid, España</t>
+  </si>
+  <si>
+    <t>47005</t>
+  </si>
+  <si>
+    <t>Calle Cid, 24, 24003 León, España</t>
+  </si>
+  <si>
+    <t>C. Santo Domingo de Silos, 1, 42002 Soria, España</t>
+  </si>
+  <si>
+    <t>Calle de la Piedad, 10, 40002 Segovia, España</t>
+  </si>
+  <si>
+    <t>40002</t>
+  </si>
+  <si>
+    <t>C. Cruz Roja, s/n, 09006 Burgos, España</t>
+  </si>
+  <si>
+    <t>C. Cruz Roja, 5, 34003 Palencia, España</t>
+  </si>
+  <si>
+    <t>34003</t>
+  </si>
+  <si>
+    <t>C. Hornos Caleros, 41, 05003 Ávila, España</t>
+  </si>
+  <si>
+    <t>05003</t>
+  </si>
+  <si>
+    <t>Plaza de Sta. Teresa de Jesus, 4, 05001 Ávila, España</t>
+  </si>
+  <si>
+    <t>C. Hernán Cortés, 42, 49021 Zamora, España</t>
+  </si>
+  <si>
+    <t>zamora@cruzroja.es</t>
+  </si>
+  <si>
+    <t>avila@cruzroja.es</t>
+  </si>
+  <si>
+    <t>segovia@cruzroja.es</t>
+  </si>
+  <si>
+    <t>burgos@cruzroja.es</t>
+  </si>
+  <si>
+    <t>palencia@cruzroja.es</t>
+  </si>
+  <si>
+    <t>valladolid@cruzroja.es</t>
+  </si>
+  <si>
+    <t>leon@cruzroja.es</t>
+  </si>
+  <si>
+    <t>soria@cruzroja.es</t>
+  </si>
+  <si>
+    <t>C. del Santuario, 4, Local 3, 47002 Valladolid</t>
+  </si>
+  <si>
+    <t>info@ssvp.es</t>
+  </si>
+  <si>
+    <t>C/ Pedro Mendoza, 11-13, bajo (local)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">37004 </t>
+  </si>
+  <si>
+    <t>sedesalamanca@apramp.org</t>
+  </si>
+  <si>
+    <t>47007</t>
+  </si>
+  <si>
+    <t>24002</t>
+  </si>
+  <si>
+    <t>34001</t>
+  </si>
+  <si>
+    <t>49003</t>
+  </si>
+  <si>
+    <t>09004</t>
+  </si>
+  <si>
+    <t>37001</t>
+  </si>
+  <si>
+    <t>C. de la India, 1, 47007 Valladolid</t>
+  </si>
+  <si>
+    <t>C. Luis Salvador Carmona, 13, 1, 24002 León</t>
+  </si>
+  <si>
+    <t>Pl. San Clemente, 7, 42002 Soria</t>
+  </si>
+  <si>
+    <t>P.º San Roque, 5-7, 05003 Ávila</t>
+  </si>
+  <si>
+    <t>C. Gil de Fuentes, 1, 34001 Palencia</t>
+  </si>
+  <si>
+    <t>C. San Atilano, 2, 49003 Zamora</t>
+  </si>
+  <si>
+    <t>Av. Acueducto, 30, 40002 Segovia</t>
+  </si>
+  <si>
+    <t>C. Vitoria, 13, 09004 Burgos</t>
+  </si>
+  <si>
+    <t>Calle Bermejeros, 14, 37001 Salamanca</t>
+  </si>
+  <si>
+    <t>Plaza la Concordia, 7 bajo. 34410 Monzón de Campos, Palencia.</t>
+  </si>
+  <si>
+    <t>34410</t>
+  </si>
+  <si>
+    <t>Monzón de Campos</t>
+  </si>
+  <si>
+    <t>C. Gaspar Arroyo, 6, 34005 Palencia</t>
+  </si>
+  <si>
+    <t>34005</t>
+  </si>
+  <si>
+    <t>coordinación@cocemfecyl.es</t>
+  </si>
+  <si>
+    <t>C. Filiberto Villalobos, 0, 37700 Béjar, Salamanca</t>
+  </si>
+  <si>
+    <t>Béjar</t>
+  </si>
+  <si>
+    <t>C. Diez Taravilla, 6, 37500 Ciudad Rodrigo, Salamanca</t>
+  </si>
+  <si>
+    <t>dmatias@caritascrodrigo.es</t>
+  </si>
+  <si>
+    <t>37500</t>
+  </si>
+  <si>
+    <t>Ciudad Rodrigo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avenida de los Cedros, 53, bajo, 37004 Salamanca </t>
+  </si>
+  <si>
+    <t>C/ Santiago nº1 ; 37008 – Salamanca</t>
+  </si>
+  <si>
+    <t>37008</t>
+  </si>
+  <si>
+    <t>fmpcastillaleon@hotmail.com</t>
+  </si>
+  <si>
+    <t>C. Arco, 2-6, 2º f, 37002 Salamanca, España</t>
+  </si>
+  <si>
+    <t>Calle Plateros, 19, bajo, 37006, Salamanca</t>
+  </si>
+  <si>
+    <t>salamanca@asecal.org</t>
+  </si>
+  <si>
+    <t>37006</t>
+  </si>
+  <si>
+    <t>Avda. San Ignacio de Loyola, 159, bajo, 24010, S. Andrés de Rabanedo, León.</t>
+  </si>
+  <si>
+    <t>leon@asecal.org</t>
+  </si>
+  <si>
+    <t>San Andres de Rabanedo</t>
+  </si>
+  <si>
+    <t>burgos@asecal.org</t>
+  </si>
+  <si>
+    <t>09001</t>
+  </si>
+  <si>
+    <t>Calle Granada, 21, 47012, Valladolid</t>
+  </si>
+  <si>
+    <t>valladolid@asecal.org</t>
+  </si>
+  <si>
+    <t>47012</t>
+  </si>
+  <si>
+    <t>C. Reina Leonor, 14, 09001 Burgos</t>
+  </si>
+  <si>
+    <t>caritas@caritasalamanca.org</t>
+  </si>
+  <si>
+    <t>C. Corrales de Monroy, 2, 37001 Salamanca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">info@asociacionplazamayor.es
+</t>
+  </si>
+  <si>
+    <t>P.º del Rector Esperabé, 6, 37008 Salamanca</t>
+  </si>
+  <si>
+    <t>info@valdecea.org</t>
+  </si>
+  <si>
+    <t>C/ Olleros 1, 47680 Mayorga (Valladolid)</t>
+  </si>
+  <si>
+    <t>47680</t>
+  </si>
+  <si>
+    <t>Mayorga</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calle Mediana, 5 – Bajo A, 47800 Medina de Rioseco (Valladolid) </t>
+  </si>
+  <si>
+    <t>47800</t>
+  </si>
+  <si>
+    <t>Medina de Rioseco</t>
+  </si>
+  <si>
+    <t>C. Mayor, nº4, 47830 Tordehumos, Valladolid</t>
+  </si>
+  <si>
+    <t>cdrsequillo@telefonica.net</t>
+  </si>
+  <si>
+    <t>47830</t>
+  </si>
+  <si>
+    <t>Tordehumos</t>
+  </si>
+  <si>
+    <t>C. Sta. María de la Cabeza, 21, Local 1, 47012 Valladolid, España</t>
+  </si>
+  <si>
+    <t>info@redincola.org</t>
+  </si>
+  <si>
+    <t>C. Olmo, 63, 47010 Valladolid, España</t>
+  </si>
+  <si>
+    <t>47010</t>
+  </si>
+  <si>
+    <t>C/ Fuente El Sol, 2. Entreplanta, 47009 – Valladolid</t>
+  </si>
+  <si>
+    <t>47009</t>
+  </si>
+  <si>
+    <t>C/ Fray Luis de León, 14. C.P.: 47002 Valladolid.</t>
+  </si>
+  <si>
+    <t>coordinacionmarta@telefonica.net</t>
+  </si>
+  <si>
+    <t>info@valladolidacoge.org</t>
+  </si>
+  <si>
+    <t>C. de Fray Luis de León, 14, 47002 Valladolid</t>
+  </si>
+  <si>
+    <t>valladolid@menesianos.org</t>
+  </si>
+  <si>
+    <t>C/ NAVA Nº 3AValladolid, 47011, Valladolid</t>
+  </si>
+  <si>
+    <t>47011</t>
+  </si>
+  <si>
+    <t>Pasaje la Marquesina, 7, 47004 Valladolid</t>
+  </si>
+  <si>
+    <t>Plaza del Dr. Marañón, 2, 47011 Valladolid</t>
+  </si>
+  <si>
+    <t>C. del Santuario, 24, 47002 Valladolid</t>
+  </si>
+  <si>
+    <t>C. Las Huertas, 6, 47140 Laguna de Duero, Valladolid</t>
+  </si>
+  <si>
+    <t>47140</t>
+  </si>
+  <si>
+    <t>Laguna de Duero</t>
+  </si>
+  <si>
+    <t>C. Félix Martín, 41, 47420 Íscar, Valladolid</t>
+  </si>
+  <si>
+    <t>47420</t>
+  </si>
+  <si>
+    <t>Íscar</t>
+  </si>
+  <si>
+    <t>Calle Almte., 32, 47400 Medina del Campo, Valladolid</t>
+  </si>
+  <si>
+    <t>47400</t>
+  </si>
+  <si>
+    <t>Medina del Campo</t>
+  </si>
+  <si>
+    <t>C. Empedrada, 20, 47800 Medina de Rioseco, Valladolid</t>
+  </si>
+  <si>
+    <t>salamanca@fundacionadsis.org</t>
+  </si>
+  <si>
+    <t>Maestro Soler 17-21, 37008 Salamanca (Salamanca)</t>
+  </si>
+  <si>
+    <t>Mirabel 9, 47003 Valladolid (Valladolid)</t>
+  </si>
+  <si>
+    <t>47003</t>
+  </si>
+  <si>
+    <t>rosachacelrosachacel.org</t>
+  </si>
+  <si>
+    <t>Plaza Santa Cruz 6 4º puerta 405, 47002 Valladolid</t>
+  </si>
+  <si>
+    <t>comunicacion@caritaszamora.org</t>
+  </si>
+  <si>
+    <t>49001</t>
+  </si>
+  <si>
+    <t>Pl. Viriato, 1, 49001 Zamora</t>
+  </si>
+  <si>
+    <t>fundaciononce@fundaciononce.es</t>
+  </si>
+  <si>
+    <t>41.650242</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.718028</t>
+  </si>
+  <si>
+    <t>40.978138</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -5.652189</t>
+  </si>
+  <si>
+    <t>40.942809</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.116448</t>
+  </si>
+  <si>
+    <t>41.765524</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -2.465487</t>
+  </si>
+  <si>
+    <t>40.654995</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.693750</t>
+  </si>
+  <si>
+    <t>42.348851</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -3.688876</t>
+  </si>
+  <si>
+    <t>42.601830</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -5.592142</t>
+  </si>
+  <si>
+    <t>40.965133</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -5.669135</t>
+  </si>
+  <si>
+    <t>41.648589</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.726044</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.726151</t>
+  </si>
+  <si>
+    <t>41.651134</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.734216</t>
+  </si>
+  <si>
+    <t>41.653507</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.713617</t>
+  </si>
+  <si>
+    <t>42.649650</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -5.538238</t>
+  </si>
+  <si>
+    <t>41.762721</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -2.465654</t>
+  </si>
+  <si>
+    <t>40.946302</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.125809</t>
+  </si>
+  <si>
+    <t>42.345857</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -3.683589</t>
+  </si>
+  <si>
+    <t>42.019761</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.527436</t>
+  </si>
+  <si>
+    <t>40.650519</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.671956</t>
+  </si>
+  <si>
+    <t>40.655553</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.696300</t>
+  </si>
+  <si>
+    <t>41.513007</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -5.726689</t>
+  </si>
+  <si>
+    <t>41.671976</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.713704</t>
+  </si>
+  <si>
+    <t>40.971603</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -5.653825</t>
+  </si>
+  <si>
+    <t>41.640262</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.732567</t>
+  </si>
+  <si>
+    <t>42.602670</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -5.576318</t>
+  </si>
+  <si>
+    <t>41.764891</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -2.466834</t>
+  </si>
+  <si>
+    <t>40.654150</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.691734</t>
+  </si>
+  <si>
+    <t>42.010125</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.534539</t>
+  </si>
+  <si>
+    <t>41.504442</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -5.744271</t>
+  </si>
+  <si>
+    <t>40.945037</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.120836</t>
+  </si>
+  <si>
+    <t>42.341629</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -3.697309</t>
+  </si>
+  <si>
+    <t>40.965690</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -5.660676</t>
+  </si>
+  <si>
+    <t>42.115708</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.495175</t>
+  </si>
+  <si>
+    <t>42.011230</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.538990</t>
+  </si>
+  <si>
+    <t>42.011325</t>
+  </si>
+  <si>
+    <t>40.598091</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -6.534964</t>
+  </si>
+  <si>
+    <t>40.974489</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -5.649794</t>
+  </si>
+  <si>
+    <t>40.958970</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -5.666816</t>
+  </si>
+  <si>
+    <t>40.969109</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -5.663268</t>
+  </si>
+  <si>
+    <t>40.975690</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -5.667962</t>
+  </si>
+  <si>
+    <t>42.610714</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -5.597049</t>
+  </si>
+  <si>
+    <t>42.337198</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -3.716298</t>
+  </si>
+  <si>
+    <t>41.642108</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.718007</t>
+  </si>
+  <si>
+    <t>40.967919</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -5.660693</t>
+  </si>
+  <si>
+    <t>40.959037</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -5.665459</t>
+  </si>
+  <si>
+    <t>42.163226</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -5.264519</t>
+  </si>
+  <si>
+    <t>41.883833</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -5.042199</t>
+  </si>
+  <si>
+    <t>41.839609</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -5.154162</t>
+  </si>
+  <si>
+    <t>41.645651</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.700269</t>
+  </si>
+  <si>
+    <t>41.663062</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.716865</t>
+  </si>
+  <si>
+    <t>41.661540</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.732798</t>
+  </si>
+  <si>
+    <t>41.650671</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.722985</t>
+  </si>
+  <si>
+    <t>41.650703</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.722438</t>
+  </si>
+  <si>
+    <t>41.646405</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.724357</t>
+  </si>
+  <si>
+    <t>41.646231</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.724293</t>
+  </si>
+  <si>
+    <t>41.658391</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.715577</t>
+  </si>
+  <si>
+    <t>41.649687</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.720655</t>
+  </si>
+  <si>
+    <t>41.581996</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.724148</t>
+  </si>
+  <si>
+    <t>41.359709</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.535748</t>
+  </si>
+  <si>
+    <t>41.309389</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.917699</t>
+  </si>
+  <si>
+    <t>41.883578</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -5.042828</t>
+  </si>
+  <si>
+    <t>40.952783</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -5.665442</t>
+  </si>
+  <si>
+    <t>41.659997</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.729106</t>
+  </si>
+  <si>
+    <t>41.651759</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.721348</t>
+  </si>
+  <si>
+    <t>41.502847</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -5.747461</t>
+  </si>
+  <si>
+    <t>42.347467</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -3.683290</t>
   </si>
 </sst>
 </file>
@@ -1284,7 +1714,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -1293,15 +1723,24 @@
   </cellStyles>
   <dxfs count="14">
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -1319,15 +1758,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -1418,18 +1848,18 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B0B80D5D-97F6-43A8-AC89-3F7237B7F48D}" name="sedes_entidades_rows" displayName="sedes_entidades_rows" ref="A1:I31" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:I31" xr:uid="{B0B80D5D-97F6-43A8-AC89-3F7237B7F48D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B0B80D5D-97F6-43A8-AC89-3F7237B7F48D}" name="sedes_entidades_rows" displayName="sedes_entidades_rows" ref="A1:I66" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:I66" xr:uid="{B0B80D5D-97F6-43A8-AC89-3F7237B7F48D}"/>
   <tableColumns count="9">
-    <tableColumn id="2" xr3:uid="{0D7B17DA-8AD2-493D-9DD5-1A671E4AF0A5}" uniqueName="2" name="entidad_id" queryTableFieldId="2" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{1D5E1CB7-1C11-4FF0-AE60-BB74F7F9022C}" uniqueName="3" name="direccion" queryTableFieldId="3" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{0D7B17DA-8AD2-493D-9DD5-1A671E4AF0A5}" uniqueName="2" name="entidad_id" queryTableFieldId="2" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{1D5E1CB7-1C11-4FF0-AE60-BB74F7F9022C}" uniqueName="3" name="direccion" queryTableFieldId="3" dataDxfId="6"/>
     <tableColumn id="4" xr3:uid="{37B9087C-0B41-42E5-8803-1D8B9F27FFA7}" uniqueName="4" name="telefono" queryTableFieldId="4"/>
-    <tableColumn id="5" xr3:uid="{BC39CA15-F0CF-409E-83A5-6FC774964ED0}" uniqueName="5" name="email" queryTableFieldId="5" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{B60F5389-BB4D-40CD-BA36-034F47D4E7A0}" uniqueName="6" name="latitud" queryTableFieldId="6" dataDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{1BA19556-8C96-40D5-A123-68DA0344B121}" uniqueName="7" name="longitud" queryTableFieldId="7" dataDxfId="0"/>
-    <tableColumn id="8" xr3:uid="{3A712945-49BE-4388-B46A-074EF8BFDD63}" uniqueName="8" name="codigo_postal" queryTableFieldId="8" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{1DA16BEB-094B-4DA9-9632-85B528BE840A}" uniqueName="9" name="municipio" queryTableFieldId="9" dataDxfId="7"/>
-    <tableColumn id="10" xr3:uid="{6897CEFB-63C7-4466-BF41-B23403EB1A9F}" uniqueName="10" name="provincia" queryTableFieldId="10" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{BC39CA15-F0CF-409E-83A5-6FC774964ED0}" uniqueName="5" name="email" queryTableFieldId="5" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{B60F5389-BB4D-40CD-BA36-034F47D4E7A0}" uniqueName="6" name="latitud" queryTableFieldId="6" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{1BA19556-8C96-40D5-A123-68DA0344B121}" uniqueName="7" name="longitud" queryTableFieldId="7" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{3A712945-49BE-4388-B46A-074EF8BFDD63}" uniqueName="8" name="codigo_postal" queryTableFieldId="8" dataDxfId="0"/>
+    <tableColumn id="9" xr3:uid="{1DA16BEB-094B-4DA9-9632-85B528BE840A}" uniqueName="9" name="municipio" queryTableFieldId="9" dataDxfId="1"/>
+    <tableColumn id="10" xr3:uid="{6897CEFB-63C7-4466-BF41-B23403EB1A9F}" uniqueName="10" name="provincia" queryTableFieldId="10" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3080,21 +3510,21 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8DD03DC-1DA1-4DA7-B875-9EE1FB7CB3BC}">
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:I66"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="66.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="68.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="33.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.42578125" style="3" customWidth="1"/>
-    <col min="6" max="6" width="12.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.7109375" style="3" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="20.85546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -3123,640 +3553,607 @@
         <v>245</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
-        <v>1</v>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>12</v>
       </c>
       <c r="B2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C2">
+        <v>983539906</v>
+      </c>
+      <c r="D2" t="s">
+        <v>260</v>
+      </c>
+      <c r="E2" t="s">
+        <v>410</v>
+      </c>
+      <c r="F2" t="s">
+        <v>411</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="H2" t="s">
+        <v>246</v>
+      </c>
+      <c r="I2" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>262</v>
+      </c>
+      <c r="C3">
+        <v>923124567</v>
+      </c>
+      <c r="D3" t="s">
+        <v>263</v>
+      </c>
+      <c r="E3" t="s">
+        <v>412</v>
+      </c>
+      <c r="F3" t="s">
+        <v>413</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="H3" t="s">
+        <v>253</v>
+      </c>
+      <c r="I3" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>264</v>
+      </c>
+      <c r="C4">
+        <v>921619985</v>
+      </c>
+      <c r="D4" t="s">
+        <v>265</v>
+      </c>
+      <c r="E4" t="s">
+        <v>414</v>
+      </c>
+      <c r="F4" t="s">
+        <v>415</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="H4" t="s">
+        <v>258</v>
+      </c>
+      <c r="I4" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>266</v>
+      </c>
+      <c r="C5">
+        <v>697163963</v>
+      </c>
+      <c r="D5" t="s">
+        <v>267</v>
+      </c>
+      <c r="E5" t="s">
+        <v>416</v>
+      </c>
+      <c r="F5" t="s">
+        <v>417</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="H5" t="s">
+        <v>256</v>
+      </c>
+      <c r="I5" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
+        <v>268</v>
+      </c>
+      <c r="C6">
+        <v>920256152</v>
+      </c>
+      <c r="D6" t="s">
+        <v>277</v>
+      </c>
+      <c r="E6" t="s">
+        <v>418</v>
+      </c>
+      <c r="F6" t="s">
+        <v>419</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="H6" t="s">
         <v>250</v>
       </c>
-      <c r="C2">
-        <v>920340332</v>
-      </c>
-      <c r="D2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" s="3">
-        <v>40.356769</v>
-      </c>
-      <c r="F2" s="3">
-        <v>-5.527094</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>253</v>
-      </c>
-      <c r="H2" t="s">
+      <c r="I6" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>269</v>
+      </c>
+      <c r="C7">
+        <v>947268620</v>
+      </c>
+      <c r="D7" t="s">
+        <v>270</v>
+      </c>
+      <c r="E7" t="s">
+        <v>420</v>
+      </c>
+      <c r="F7" t="s">
+        <v>421</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="I2" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>254</v>
-      </c>
-      <c r="C3">
-        <v>947244914</v>
-      </c>
-      <c r="D3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" s="3">
-        <v>42.357402</v>
-      </c>
-      <c r="F3" s="3">
-        <v>-3.6707190000000001</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>255</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="H7" t="s">
         <v>248</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I7" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>256</v>
-      </c>
-      <c r="C4">
-        <v>947232303</v>
-      </c>
-      <c r="D4" t="s">
-        <v>23</v>
-      </c>
-      <c r="E4" s="3">
-        <v>42.351576999999999</v>
-      </c>
-      <c r="F4" s="3">
-        <v>-3.6928040000000002</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>255</v>
-      </c>
-      <c r="H4" t="s">
-        <v>248</v>
-      </c>
-      <c r="I4" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>257</v>
-      </c>
-      <c r="C5">
-        <v>947232303</v>
-      </c>
-      <c r="D5" t="s">
-        <v>23</v>
-      </c>
-      <c r="E5" s="3">
-        <v>42.353344</v>
-      </c>
-      <c r="F5" s="3">
-        <v>3.6815579999999999</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>255</v>
-      </c>
-      <c r="H5" t="s">
-        <v>248</v>
-      </c>
-      <c r="I5" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
-        <v>4</v>
-      </c>
-      <c r="B6" t="s">
-        <v>258</v>
-      </c>
-      <c r="C6">
-        <v>947214343</v>
-      </c>
-      <c r="D6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E6" s="3">
-        <v>42.349418</v>
-      </c>
-      <c r="F6" s="3">
-        <v>-3.6809880000000001</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>255</v>
-      </c>
-      <c r="H6" t="s">
-        <v>248</v>
-      </c>
-      <c r="I6" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
-        <v>5</v>
-      </c>
-      <c r="B7" t="s">
-        <v>259</v>
-      </c>
-      <c r="C7">
-        <v>987387119</v>
-      </c>
-      <c r="D7" t="s">
-        <v>284</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>349</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>350</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>266</v>
-      </c>
-      <c r="H7" t="s">
-        <v>260</v>
-      </c>
-      <c r="I7" t="s">
-        <v>247</v>
-      </c>
-      <c r="K7" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="2">
-        <v>5</v>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>261</v>
+        <v>271</v>
       </c>
       <c r="C8">
-        <v>987410324</v>
+        <v>987876143</v>
       </c>
       <c r="D8" t="s">
-        <v>284</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>351</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>352</v>
+        <v>75</v>
+      </c>
+      <c r="E8" t="s">
+        <v>422</v>
+      </c>
+      <c r="F8" t="s">
+        <v>423</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="H8" t="s">
-        <v>262</v>
+        <v>276</v>
       </c>
       <c r="I8" t="s">
         <v>247</v>
       </c>
-      <c r="K8" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="2">
-        <v>5</v>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>263</v>
+        <v>278</v>
       </c>
       <c r="C9">
-        <v>987427500</v>
+        <v>923314142</v>
       </c>
       <c r="D9" t="s">
+        <v>279</v>
+      </c>
+      <c r="E9" t="s">
+        <v>424</v>
+      </c>
+      <c r="F9" t="s">
+        <v>425</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="H9" t="s">
+        <v>253</v>
+      </c>
+      <c r="I9" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>13</v>
+      </c>
+      <c r="B10" t="s">
+        <v>281</v>
+      </c>
+      <c r="C10" s="3">
+        <v>661260040</v>
+      </c>
+      <c r="D10" t="s">
+        <v>282</v>
+      </c>
+      <c r="E10" t="s">
+        <v>426</v>
+      </c>
+      <c r="F10" t="s">
+        <v>427</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="H10" t="s">
+        <v>256</v>
+      </c>
+      <c r="I10" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>13</v>
+      </c>
+      <c r="B11" t="s">
         <v>284</v>
       </c>
-      <c r="E9" s="3" t="s">
-        <v>353</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>354</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>267</v>
-      </c>
-      <c r="H9" t="s">
-        <v>262</v>
-      </c>
-      <c r="I9" t="s">
+      <c r="C11">
+        <v>637763255</v>
+      </c>
+      <c r="D11" t="s">
+        <v>285</v>
+      </c>
+      <c r="E11" t="s">
+        <v>426</v>
+      </c>
+      <c r="F11" t="s">
+        <v>428</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="H11" t="s">
+        <v>246</v>
+      </c>
+      <c r="I11" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>14</v>
+      </c>
+      <c r="B12" t="s">
+        <v>287</v>
+      </c>
+      <c r="C12">
+        <v>983336777</v>
+      </c>
+      <c r="D12" t="s">
+        <v>307</v>
+      </c>
+      <c r="E12" t="s">
+        <v>429</v>
+      </c>
+      <c r="F12" t="s">
+        <v>430</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="H12" t="s">
+        <v>246</v>
+      </c>
+      <c r="I12" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>14</v>
+      </c>
+      <c r="B13" t="s">
+        <v>289</v>
+      </c>
+      <c r="C13">
+        <v>983132828</v>
+      </c>
+      <c r="D13" t="s">
+        <v>307</v>
+      </c>
+      <c r="E13" t="s">
+        <v>431</v>
+      </c>
+      <c r="F13" t="s">
+        <v>432</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="H13" t="s">
+        <v>246</v>
+      </c>
+      <c r="I13" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>14</v>
+      </c>
+      <c r="B14" t="s">
+        <v>291</v>
+      </c>
+      <c r="C14">
+        <v>987252535</v>
+      </c>
+      <c r="D14" t="s">
+        <v>308</v>
+      </c>
+      <c r="E14" t="s">
+        <v>433</v>
+      </c>
+      <c r="F14" t="s">
+        <v>434</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="H14" t="s">
         <v>247</v>
-      </c>
-      <c r="K9" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="2">
-        <v>5</v>
-      </c>
-      <c r="B10" t="s">
-        <v>264</v>
-      </c>
-      <c r="C10">
-        <v>987511678</v>
-      </c>
-      <c r="D10" t="s">
-        <v>284</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>355</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>356</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>268</v>
-      </c>
-      <c r="H10" t="s">
-        <v>265</v>
-      </c>
-      <c r="I10" t="s">
-        <v>247</v>
-      </c>
-      <c r="K10" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="2">
-        <v>5</v>
-      </c>
-      <c r="B11" t="s">
-        <v>269</v>
-      </c>
-      <c r="C11">
-        <v>987656721</v>
-      </c>
-      <c r="D11" t="s">
-        <v>284</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>357</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>358</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>270</v>
-      </c>
-      <c r="H11" t="s">
-        <v>271</v>
-      </c>
-      <c r="I11" t="s">
-        <v>247</v>
-      </c>
-      <c r="K11" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="2">
-        <v>5</v>
-      </c>
-      <c r="B12" t="s">
-        <v>272</v>
-      </c>
-      <c r="C12">
-        <v>988320933</v>
-      </c>
-      <c r="D12" t="s">
-        <v>284</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>359</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>360</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>273</v>
-      </c>
-      <c r="H12" t="s">
-        <v>274</v>
-      </c>
-      <c r="I12" t="s">
-        <v>247</v>
-      </c>
-      <c r="K12" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="2">
-        <v>5</v>
-      </c>
-      <c r="B13" t="s">
-        <v>275</v>
-      </c>
-      <c r="C13">
-        <v>698152864</v>
-      </c>
-      <c r="D13" t="s">
-        <v>284</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>361</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>362</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="H13" t="s">
-        <v>277</v>
-      </c>
-      <c r="I13" t="s">
-        <v>247</v>
-      </c>
-      <c r="K13" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="2">
-        <v>5</v>
-      </c>
-      <c r="B14" t="s">
-        <v>278</v>
-      </c>
-      <c r="C14">
-        <v>698152864</v>
-      </c>
-      <c r="D14" t="s">
-        <v>284</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>363</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>364</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="H14" t="s">
-        <v>280</v>
       </c>
       <c r="I14" t="s">
         <v>247</v>
       </c>
-      <c r="K14" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="2">
-        <v>5</v>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>281</v>
+        <v>292</v>
       </c>
       <c r="C15">
-        <v>622824314</v>
+        <v>975212640</v>
       </c>
       <c r="D15" t="s">
-        <v>284</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>365</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>366</v>
+        <v>309</v>
+      </c>
+      <c r="E15" t="s">
+        <v>435</v>
+      </c>
+      <c r="F15" t="s">
+        <v>436</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>282</v>
+        <v>272</v>
       </c>
       <c r="H15" t="s">
-        <v>283</v>
+        <v>256</v>
       </c>
       <c r="I15" t="s">
-        <v>247</v>
-      </c>
-      <c r="K15" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" s="2">
-        <v>6</v>
+        <v>256</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>285</v>
+        <v>293</v>
       </c>
       <c r="C16">
-        <v>987388737</v>
+        <v>921440202</v>
       </c>
       <c r="D16" t="s">
-        <v>41</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>367</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>368</v>
+        <v>304</v>
+      </c>
+      <c r="E16" t="s">
+        <v>437</v>
+      </c>
+      <c r="F16" t="s">
+        <v>438</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>286</v>
+        <v>294</v>
       </c>
       <c r="H16" t="s">
-        <v>287</v>
+        <v>258</v>
       </c>
       <c r="I16" t="s">
-        <v>247</v>
-      </c>
-      <c r="K16" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" s="2">
-        <v>8</v>
+        <v>258</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>14</v>
       </c>
       <c r="B17" t="s">
-        <v>288</v>
+        <v>295</v>
       </c>
       <c r="C17">
-        <v>987218617</v>
+        <v>947212311</v>
       </c>
       <c r="D17" t="s">
-        <v>53</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>369</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>370</v>
+        <v>305</v>
+      </c>
+      <c r="E17" t="s">
+        <v>439</v>
+      </c>
+      <c r="F17" t="s">
+        <v>440</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>289</v>
+        <v>251</v>
       </c>
       <c r="H17" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="I17" t="s">
-        <v>247</v>
-      </c>
-      <c r="K17" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A18" s="2">
-        <v>9</v>
+        <v>248</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>14</v>
       </c>
       <c r="B18" t="s">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="C18">
-        <v>987105110</v>
-      </c>
-      <c r="E18" s="3">
-        <v>42.584688999999997</v>
-      </c>
-      <c r="F18" s="3">
-        <v>-5.5673389999999996</v>
+        <v>979700507</v>
+      </c>
+      <c r="D18" t="s">
+        <v>306</v>
+      </c>
+      <c r="E18" t="s">
+        <v>441</v>
+      </c>
+      <c r="F18" t="s">
+        <v>442</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="H18" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="I18" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" s="2">
-        <v>9</v>
+        <v>249</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>14</v>
       </c>
       <c r="B19" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="C19">
-        <v>987049556</v>
-      </c>
-      <c r="E19" s="3">
-        <v>42.557397000000002</v>
-      </c>
-      <c r="F19" s="3">
-        <v>-6.5997820000000003</v>
+        <v>920224848</v>
+      </c>
+      <c r="D19" t="s">
+        <v>303</v>
+      </c>
+      <c r="E19" t="s">
+        <v>443</v>
+      </c>
+      <c r="F19" t="s">
+        <v>444</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>293</v>
+        <v>299</v>
       </c>
       <c r="H19" t="s">
-        <v>262</v>
+        <v>250</v>
       </c>
       <c r="I19" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" s="2">
-        <v>10</v>
+        <v>250</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>14</v>
       </c>
       <c r="B20" t="s">
-        <v>294</v>
+        <v>300</v>
       </c>
       <c r="C20">
-        <v>923244262</v>
+        <v>920213248</v>
       </c>
       <c r="D20" t="s">
-        <v>295</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>371</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>372</v>
+        <v>303</v>
+      </c>
+      <c r="E20" t="s">
+        <v>445</v>
+      </c>
+      <c r="F20" t="s">
+        <v>446</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>297</v>
+        <v>274</v>
       </c>
       <c r="H20" t="s">
-        <v>296</v>
+        <v>250</v>
       </c>
       <c r="I20" t="s">
-        <v>296</v>
-      </c>
-      <c r="K20" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A21" s="2">
-        <v>10</v>
+        <v>250</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>14</v>
       </c>
       <c r="B21" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="C21">
-        <v>923244262</v>
+        <v>980523300</v>
       </c>
       <c r="D21" t="s">
-        <v>295</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>373</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>374</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>297</v>
+        <v>302</v>
+      </c>
+      <c r="E21" t="s">
+        <v>447</v>
+      </c>
+      <c r="F21" t="s">
+        <v>448</v>
+      </c>
+      <c r="G21" s="1">
+        <v>49021</v>
       </c>
       <c r="H21" t="s">
-        <v>296</v>
+        <v>257</v>
       </c>
       <c r="I21" t="s">
-        <v>296</v>
-      </c>
-      <c r="K21" t="s">
-        <v>336</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22" s="2">
-        <v>10</v>
+        <v>257</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>15</v>
       </c>
       <c r="B22" t="s">
-        <v>299</v>
+        <v>310</v>
       </c>
       <c r="C22">
-        <v>983399643</v>
+        <v>983298269</v>
       </c>
       <c r="D22" t="s">
-        <v>300</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>375</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>376</v>
+        <v>311</v>
+      </c>
+      <c r="E22" t="s">
+        <v>449</v>
+      </c>
+      <c r="F22" t="s">
+        <v>450</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>301</v>
+        <v>261</v>
       </c>
       <c r="H22" t="s">
         <v>246</v>
@@ -3764,176 +4161,173 @@
       <c r="I22" t="s">
         <v>246</v>
       </c>
-      <c r="K22" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A23" s="2">
-        <v>10</v>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>16</v>
       </c>
       <c r="B23" t="s">
-        <v>302</v>
+        <v>312</v>
       </c>
       <c r="C23">
-        <v>975679125</v>
+        <v>923229835</v>
       </c>
       <c r="D23" t="s">
-        <v>303</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>377</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>378</v>
+        <v>314</v>
+      </c>
+      <c r="E23" t="s">
+        <v>451</v>
+      </c>
+      <c r="F23" t="s">
+        <v>452</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>304</v>
+        <v>313</v>
       </c>
       <c r="H23" t="s">
-        <v>305</v>
+        <v>253</v>
       </c>
       <c r="I23" t="s">
-        <v>306</v>
-      </c>
-      <c r="K23" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A24" s="2">
-        <v>11</v>
+        <v>253</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>17</v>
       </c>
       <c r="B24" t="s">
-        <v>307</v>
+        <v>321</v>
       </c>
       <c r="C24">
-        <v>923280985</v>
+        <v>983300888</v>
       </c>
       <c r="D24" t="s">
-        <v>308</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>379</v>
-      </c>
-      <c r="F24" s="3" t="s">
-        <v>380</v>
+        <v>409</v>
+      </c>
+      <c r="E24" t="s">
+        <v>453</v>
+      </c>
+      <c r="F24" t="s">
+        <v>454</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>315</v>
       </c>
       <c r="H24" t="s">
-        <v>296</v>
+        <v>246</v>
       </c>
       <c r="I24" t="s">
-        <v>296</v>
-      </c>
-      <c r="K24" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A25" s="2">
-        <v>11</v>
+        <v>246</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>18</v>
       </c>
       <c r="B25" t="s">
-        <v>309</v>
+        <v>322</v>
       </c>
       <c r="C25">
-        <v>676986948</v>
+        <v>987875390</v>
       </c>
       <c r="D25" t="s">
-        <v>310</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>381</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>382</v>
+        <v>409</v>
+      </c>
+      <c r="E25" t="s">
+        <v>455</v>
+      </c>
+      <c r="F25" t="s">
+        <v>456</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>316</v>
       </c>
       <c r="H25" t="s">
-        <v>311</v>
+        <v>247</v>
       </c>
       <c r="I25" t="s">
-        <v>248</v>
-      </c>
-      <c r="K25" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A26" s="2">
-        <v>11</v>
+        <v>247</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>18</v>
       </c>
       <c r="B26" t="s">
-        <v>312</v>
+        <v>323</v>
       </c>
       <c r="C26">
-        <v>947242425</v>
+        <v>975254570</v>
       </c>
       <c r="D26" t="s">
-        <v>313</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>383</v>
-      </c>
-      <c r="F26" s="3" t="s">
-        <v>384</v>
+        <v>409</v>
+      </c>
+      <c r="E26" t="s">
+        <v>457</v>
+      </c>
+      <c r="F26" t="s">
+        <v>458</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>272</v>
       </c>
       <c r="H26" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="I26" t="s">
-        <v>248</v>
-      </c>
-      <c r="K26" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A27" s="2">
-        <v>11</v>
+        <v>256</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>18</v>
       </c>
       <c r="B27" t="s">
-        <v>314</v>
+        <v>324</v>
       </c>
       <c r="C27">
-        <v>987276600</v>
+        <v>920312752</v>
       </c>
       <c r="D27" t="s">
-        <v>315</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>385</v>
-      </c>
-      <c r="F27" s="3" t="s">
-        <v>386</v>
+        <v>409</v>
+      </c>
+      <c r="E27" t="s">
+        <v>459</v>
+      </c>
+      <c r="F27" t="s">
+        <v>460</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>299</v>
       </c>
       <c r="H27" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="I27" t="s">
-        <v>247</v>
-      </c>
-      <c r="K27" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A28" s="2">
-        <v>11</v>
+        <v>250</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>18</v>
       </c>
       <c r="B28" t="s">
-        <v>344</v>
+        <v>325</v>
       </c>
       <c r="C28">
-        <v>979706073</v>
+        <v>979706582</v>
       </c>
       <c r="D28" t="s">
-        <v>316</v>
-      </c>
-      <c r="E28" s="3" t="s">
-        <v>387</v>
-      </c>
-      <c r="F28" s="3" t="s">
-        <v>388</v>
+        <v>409</v>
+      </c>
+      <c r="E28" t="s">
+        <v>461</v>
+      </c>
+      <c r="F28" t="s">
+        <v>462</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>317</v>
       </c>
       <c r="H28" t="s">
         <v>249</v>
@@ -3941,101 +4335,1171 @@
       <c r="I28" t="s">
         <v>249</v>
       </c>
-      <c r="K28" t="s">
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>18</v>
+      </c>
+      <c r="B29" t="s">
+        <v>326</v>
+      </c>
+      <c r="C29">
+        <v>980697583</v>
+      </c>
+      <c r="D29" t="s">
+        <v>409</v>
+      </c>
+      <c r="E29" t="s">
+        <v>463</v>
+      </c>
+      <c r="F29" t="s">
+        <v>464</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="H29" t="s">
+        <v>257</v>
+      </c>
+      <c r="I29" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>18</v>
+      </c>
+      <c r="B30" t="s">
+        <v>327</v>
+      </c>
+      <c r="C30">
+        <v>921461621</v>
+      </c>
+      <c r="D30" t="s">
+        <v>409</v>
+      </c>
+      <c r="E30" t="s">
+        <v>465</v>
+      </c>
+      <c r="F30" t="s">
+        <v>466</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="H30" t="s">
+        <v>258</v>
+      </c>
+      <c r="I30" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>18</v>
+      </c>
+      <c r="B31" t="s">
+        <v>328</v>
+      </c>
+      <c r="C31">
+        <v>947203861</v>
+      </c>
+      <c r="D31" t="s">
+        <v>409</v>
+      </c>
+      <c r="E31" t="s">
+        <v>467</v>
+      </c>
+      <c r="F31" t="s">
+        <v>468</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="H31" t="s">
+        <v>248</v>
+      </c>
+      <c r="I31" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>18</v>
+      </c>
+      <c r="B32" t="s">
+        <v>329</v>
+      </c>
+      <c r="C32">
+        <v>923217008</v>
+      </c>
+      <c r="D32" t="s">
+        <v>409</v>
+      </c>
+      <c r="E32" t="s">
+        <v>469</v>
+      </c>
+      <c r="F32" t="s">
+        <v>470</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="H32" t="s">
+        <v>253</v>
+      </c>
+      <c r="I32" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>19</v>
+      </c>
+      <c r="B33" t="s">
+        <v>330</v>
+      </c>
+      <c r="C33">
+        <v>979808800</v>
+      </c>
+      <c r="D33" t="s">
+        <v>115</v>
+      </c>
+      <c r="E33" t="s">
+        <v>471</v>
+      </c>
+      <c r="F33" t="s">
+        <v>472</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="H33" t="s">
+        <v>332</v>
+      </c>
+      <c r="I33" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>20</v>
+      </c>
+      <c r="B34" t="s">
+        <v>333</v>
+      </c>
+      <c r="C34">
+        <v>979745840</v>
+      </c>
+      <c r="D34" t="s">
+        <v>335</v>
+      </c>
+      <c r="E34" t="s">
+        <v>473</v>
+      </c>
+      <c r="F34" t="s">
+        <v>474</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="H34" t="s">
+        <v>249</v>
+      </c>
+      <c r="I34" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>21</v>
+      </c>
+      <c r="B35" t="s">
+        <v>336</v>
+      </c>
+      <c r="C35">
+        <v>923402270</v>
+      </c>
+      <c r="D35" t="s">
+        <v>122</v>
+      </c>
+      <c r="E35" t="s">
+        <v>475</v>
+      </c>
+      <c r="F35" t="s">
+        <v>474</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="H35" t="s">
+        <v>337</v>
+      </c>
+      <c r="I35" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>22</v>
+      </c>
+      <c r="B36" t="s">
+        <v>338</v>
+      </c>
+      <c r="C36">
+        <v>923460693</v>
+      </c>
+      <c r="D36" t="s">
+        <v>339</v>
+      </c>
+      <c r="E36" t="s">
+        <v>476</v>
+      </c>
+      <c r="F36" t="s">
+        <v>477</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="H36" t="s">
+        <v>341</v>
+      </c>
+      <c r="I36" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>23</v>
+      </c>
+      <c r="B37" t="s">
+        <v>342</v>
+      </c>
+      <c r="C37">
+        <v>923019030</v>
+      </c>
+      <c r="D37" t="s">
+        <v>131</v>
+      </c>
+      <c r="E37" t="s">
+        <v>478</v>
+      </c>
+      <c r="F37" t="s">
+        <v>479</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="H37" t="s">
+        <v>253</v>
+      </c>
+      <c r="I37" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>24</v>
+      </c>
+      <c r="B38" t="s">
+        <v>343</v>
+      </c>
+      <c r="C38">
+        <v>923219511</v>
+      </c>
+      <c r="D38" t="s">
+        <v>137</v>
+      </c>
+      <c r="E38" t="s">
+        <v>480</v>
+      </c>
+      <c r="F38" t="s">
+        <v>481</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="H38" t="s">
+        <v>253</v>
+      </c>
+      <c r="I38" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>25</v>
+      </c>
+      <c r="B39" t="s">
+        <v>346</v>
+      </c>
+      <c r="C39">
+        <v>923211900</v>
+      </c>
+      <c r="D39" t="s">
         <v>345</v>
       </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A29" s="2">
-        <v>11</v>
-      </c>
-      <c r="B29" t="s">
-        <v>317</v>
-      </c>
-      <c r="C29">
-        <v>983219622</v>
-      </c>
-      <c r="D29" t="s">
-        <v>318</v>
-      </c>
-      <c r="E29" s="3" t="s">
+      <c r="E39" t="s">
+        <v>482</v>
+      </c>
+      <c r="F39" t="s">
+        <v>483</v>
+      </c>
+      <c r="G39" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="H39" t="s">
+        <v>253</v>
+      </c>
+      <c r="I39" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>26</v>
+      </c>
+      <c r="B40" t="s">
+        <v>347</v>
+      </c>
+      <c r="C40">
+        <v>923121354</v>
+      </c>
+      <c r="D40" t="s">
+        <v>348</v>
+      </c>
+      <c r="E40" t="s">
+        <v>484</v>
+      </c>
+      <c r="F40" t="s">
+        <v>485</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="H40" t="s">
+        <v>253</v>
+      </c>
+      <c r="I40" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>26</v>
+      </c>
+      <c r="B41" t="s">
+        <v>350</v>
+      </c>
+      <c r="C41">
+        <v>987224045</v>
+      </c>
+      <c r="D41" t="s">
+        <v>351</v>
+      </c>
+      <c r="E41" t="s">
+        <v>486</v>
+      </c>
+      <c r="F41" t="s">
+        <v>487</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="H41" t="s">
+        <v>352</v>
+      </c>
+      <c r="I41" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>26</v>
+      </c>
+      <c r="B42" t="s">
+        <v>358</v>
+      </c>
+      <c r="C42">
+        <v>947279762</v>
+      </c>
+      <c r="D42" t="s">
+        <v>353</v>
+      </c>
+      <c r="E42" t="s">
+        <v>488</v>
+      </c>
+      <c r="F42" t="s">
+        <v>489</v>
+      </c>
+      <c r="G42" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="H42" t="s">
+        <v>248</v>
+      </c>
+      <c r="I42" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>26</v>
+      </c>
+      <c r="B43" t="s">
+        <v>355</v>
+      </c>
+      <c r="C43">
+        <v>983205530</v>
+      </c>
+      <c r="D43" t="s">
+        <v>356</v>
+      </c>
+      <c r="E43" t="s">
+        <v>490</v>
+      </c>
+      <c r="F43" t="s">
+        <v>491</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>357</v>
+      </c>
+      <c r="H43" t="s">
+        <v>246</v>
+      </c>
+      <c r="I43" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>27</v>
+      </c>
+      <c r="B44" t="s">
+        <v>360</v>
+      </c>
+      <c r="C44">
+        <v>923269698</v>
+      </c>
+      <c r="D44" t="s">
+        <v>359</v>
+      </c>
+      <c r="E44" t="s">
+        <v>492</v>
+      </c>
+      <c r="F44" t="s">
+        <v>493</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="H44" t="s">
+        <v>253</v>
+      </c>
+      <c r="I44" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>28</v>
+      </c>
+      <c r="B45" t="s">
+        <v>362</v>
+      </c>
+      <c r="C45">
+        <v>923211900</v>
+      </c>
+      <c r="D45" t="s">
+        <v>361</v>
+      </c>
+      <c r="E45" t="s">
+        <v>494</v>
+      </c>
+      <c r="F45" t="s">
+        <v>495</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="H45" t="s">
+        <v>253</v>
+      </c>
+      <c r="I45" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>29</v>
+      </c>
+      <c r="B46" t="s">
+        <v>364</v>
+      </c>
+      <c r="C46">
+        <v>983751568</v>
+      </c>
+      <c r="D46" t="s">
+        <v>363</v>
+      </c>
+      <c r="E46" t="s">
+        <v>496</v>
+      </c>
+      <c r="F46" t="s">
+        <v>497</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="H46" t="s">
+        <v>366</v>
+      </c>
+      <c r="I46" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>30</v>
+      </c>
+      <c r="B47" t="s">
+        <v>367</v>
+      </c>
+      <c r="C47">
+        <v>983725000</v>
+      </c>
+      <c r="D47" t="s">
+        <v>167</v>
+      </c>
+      <c r="E47" t="s">
+        <v>498</v>
+      </c>
+      <c r="F47" t="s">
+        <v>499</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="H47" t="s">
+        <v>369</v>
+      </c>
+      <c r="I47" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>31</v>
+      </c>
+      <c r="B48" t="s">
+        <v>370</v>
+      </c>
+      <c r="C48">
+        <v>983714586</v>
+      </c>
+      <c r="D48" t="s">
+        <v>371</v>
+      </c>
+      <c r="E48" t="s">
+        <v>500</v>
+      </c>
+      <c r="F48" t="s">
+        <v>501</v>
+      </c>
+      <c r="G48" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="H48" t="s">
+        <v>373</v>
+      </c>
+      <c r="I48" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>32</v>
+      </c>
+      <c r="B49" t="s">
+        <v>374</v>
+      </c>
+      <c r="C49">
+        <v>983086580</v>
+      </c>
+      <c r="D49" t="s">
+        <v>177</v>
+      </c>
+      <c r="E49" t="s">
+        <v>502</v>
+      </c>
+      <c r="F49" t="s">
+        <v>503</v>
+      </c>
+      <c r="G49" s="1" t="s">
+        <v>357</v>
+      </c>
+      <c r="H49" t="s">
+        <v>246</v>
+      </c>
+      <c r="I49" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>33</v>
+      </c>
+      <c r="B50" t="s">
+        <v>376</v>
+      </c>
+      <c r="C50">
+        <v>983307083</v>
+      </c>
+      <c r="D50" t="s">
+        <v>375</v>
+      </c>
+      <c r="E50" t="s">
+        <v>504</v>
+      </c>
+      <c r="F50" t="s">
+        <v>505</v>
+      </c>
+      <c r="G50" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="H50" t="s">
+        <v>246</v>
+      </c>
+      <c r="I50" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>34</v>
+      </c>
+      <c r="B51" t="s">
+        <v>378</v>
+      </c>
+      <c r="C51">
+        <v>983371279</v>
+      </c>
+      <c r="D51" t="s">
+        <v>189</v>
+      </c>
+      <c r="E51" t="s">
+        <v>506</v>
+      </c>
+      <c r="F51" t="s">
+        <v>507</v>
+      </c>
+      <c r="G51" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="H51" t="s">
+        <v>246</v>
+      </c>
+      <c r="I51" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>35</v>
+      </c>
+      <c r="B52" t="s">
+        <v>380</v>
+      </c>
+      <c r="C52">
+        <v>983309915</v>
+      </c>
+      <c r="D52" t="s">
+        <v>381</v>
+      </c>
+      <c r="E52" t="s">
+        <v>508</v>
+      </c>
+      <c r="F52" t="s">
+        <v>509</v>
+      </c>
+      <c r="G52" s="1">
+        <v>47002</v>
+      </c>
+      <c r="H52" t="s">
+        <v>246</v>
+      </c>
+      <c r="I52" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>36</v>
+      </c>
+      <c r="B53" t="s">
+        <v>383</v>
+      </c>
+      <c r="C53">
+        <v>983309915</v>
+      </c>
+      <c r="D53" t="s">
+        <v>382</v>
+      </c>
+      <c r="E53" t="s">
+        <v>510</v>
+      </c>
+      <c r="F53" t="s">
+        <v>511</v>
+      </c>
+      <c r="G53" s="1">
+        <v>47002</v>
+      </c>
+      <c r="H53" t="s">
+        <v>246</v>
+      </c>
+      <c r="I53" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>37</v>
+      </c>
+      <c r="B54" t="s">
+        <v>385</v>
+      </c>
+      <c r="C54">
+        <v>983251928</v>
+      </c>
+      <c r="D54" t="s">
+        <v>384</v>
+      </c>
+      <c r="E54" t="s">
+        <v>512</v>
+      </c>
+      <c r="F54" t="s">
+        <v>513</v>
+      </c>
+      <c r="G54" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="H54" t="s">
+        <v>246</v>
+      </c>
+      <c r="I54" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>38</v>
+      </c>
+      <c r="B55" t="s">
+        <v>387</v>
+      </c>
+      <c r="C55">
+        <v>983507177</v>
+      </c>
+      <c r="D55" t="s">
+        <v>208</v>
+      </c>
+      <c r="E55" t="s">
+        <v>514</v>
+      </c>
+      <c r="F55" t="s">
+        <v>515</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="H55" t="s">
+        <v>246</v>
+      </c>
+      <c r="I55" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>39</v>
+      </c>
+      <c r="B56" t="s">
+        <v>388</v>
+      </c>
+      <c r="C56">
+        <v>983202301</v>
+      </c>
+      <c r="D56" t="s">
+        <v>213</v>
+      </c>
+      <c r="E56" t="s">
+        <v>516</v>
+      </c>
+      <c r="F56" t="s">
+        <v>517</v>
+      </c>
+      <c r="G56" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="H56" t="s">
+        <v>246</v>
+      </c>
+      <c r="I56" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>39</v>
+      </c>
+      <c r="B57" t="s">
         <v>389</v>
       </c>
-      <c r="F29" s="3" t="s">
+      <c r="C57">
+        <v>983202301</v>
+      </c>
+      <c r="D57" t="s">
+        <v>213</v>
+      </c>
+      <c r="E57" t="s">
+        <v>518</v>
+      </c>
+      <c r="F57" t="s">
+        <v>519</v>
+      </c>
+      <c r="G57" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="H57" t="s">
+        <v>246</v>
+      </c>
+      <c r="I57" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>39</v>
+      </c>
+      <c r="B58" t="s">
         <v>390</v>
       </c>
-      <c r="H29" t="s">
+      <c r="C58">
+        <v>983541388</v>
+      </c>
+      <c r="D58" t="s">
+        <v>213</v>
+      </c>
+      <c r="E58" t="s">
+        <v>520</v>
+      </c>
+      <c r="F58" t="s">
+        <v>521</v>
+      </c>
+      <c r="G58" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="H58" t="s">
+        <v>392</v>
+      </c>
+      <c r="I58" t="s">
         <v>246</v>
       </c>
-      <c r="I29" t="s">
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>39</v>
+      </c>
+      <c r="B59" t="s">
+        <v>393</v>
+      </c>
+      <c r="C59">
+        <v>983620530</v>
+      </c>
+      <c r="D59" t="s">
+        <v>213</v>
+      </c>
+      <c r="E59" t="s">
+        <v>522</v>
+      </c>
+      <c r="F59" t="s">
+        <v>523</v>
+      </c>
+      <c r="G59" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="H59" t="s">
+        <v>395</v>
+      </c>
+      <c r="I59" t="s">
         <v>246</v>
       </c>
-      <c r="K29" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A30" s="2">
-        <v>11</v>
-      </c>
-      <c r="B30" t="s">
-        <v>319</v>
-      </c>
-      <c r="C30">
-        <v>980512727</v>
-      </c>
-      <c r="D30" t="s">
-        <v>320</v>
-      </c>
-      <c r="E30" s="3" t="s">
-        <v>391</v>
-      </c>
-      <c r="F30" s="3" t="s">
-        <v>392</v>
-      </c>
-      <c r="H30" t="s">
-        <v>321</v>
-      </c>
-      <c r="I30" t="s">
-        <v>321</v>
-      </c>
-      <c r="K30" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A31" s="2">
-        <v>11</v>
-      </c>
-      <c r="B31" t="s">
-        <v>347</v>
-      </c>
-      <c r="C31">
-        <v>921435241</v>
-      </c>
-      <c r="D31" t="s">
-        <v>322</v>
-      </c>
-      <c r="E31" s="3" t="s">
-        <v>393</v>
-      </c>
-      <c r="F31" s="3" t="s">
-        <v>394</v>
-      </c>
-      <c r="H31" t="s">
-        <v>323</v>
-      </c>
-      <c r="I31" t="s">
-        <v>323</v>
-      </c>
-      <c r="K31" t="s">
-        <v>348</v>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>39</v>
+      </c>
+      <c r="B60" t="s">
+        <v>396</v>
+      </c>
+      <c r="C60">
+        <v>983803118</v>
+      </c>
+      <c r="D60" t="s">
+        <v>213</v>
+      </c>
+      <c r="E60" t="s">
+        <v>524</v>
+      </c>
+      <c r="F60" t="s">
+        <v>525</v>
+      </c>
+      <c r="G60" s="1" t="s">
+        <v>397</v>
+      </c>
+      <c r="H60" t="s">
+        <v>398</v>
+      </c>
+      <c r="I60" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>39</v>
+      </c>
+      <c r="B61" t="s">
+        <v>399</v>
+      </c>
+      <c r="C61">
+        <v>983701251</v>
+      </c>
+      <c r="D61" t="s">
+        <v>213</v>
+      </c>
+      <c r="E61" t="s">
+        <v>526</v>
+      </c>
+      <c r="F61" t="s">
+        <v>527</v>
+      </c>
+      <c r="G61" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="H61" t="s">
+        <v>369</v>
+      </c>
+      <c r="I61" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>40</v>
+      </c>
+      <c r="B62" t="s">
+        <v>401</v>
+      </c>
+      <c r="C62">
+        <v>923271226</v>
+      </c>
+      <c r="D62" t="s">
+        <v>400</v>
+      </c>
+      <c r="E62" t="s">
+        <v>528</v>
+      </c>
+      <c r="F62" t="s">
+        <v>529</v>
+      </c>
+      <c r="G62" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="H62" t="s">
+        <v>253</v>
+      </c>
+      <c r="I62" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>40</v>
+      </c>
+      <c r="B63" t="s">
+        <v>402</v>
+      </c>
+      <c r="C63">
+        <v>983378285</v>
+      </c>
+      <c r="D63" t="s">
+        <v>217</v>
+      </c>
+      <c r="E63" t="s">
+        <v>530</v>
+      </c>
+      <c r="F63" t="s">
+        <v>531</v>
+      </c>
+      <c r="G63" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="H63" t="s">
+        <v>246</v>
+      </c>
+      <c r="I63" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>41</v>
+      </c>
+      <c r="B64" t="s">
+        <v>405</v>
+      </c>
+      <c r="C64">
+        <v>983397325</v>
+      </c>
+      <c r="D64" t="s">
+        <v>404</v>
+      </c>
+      <c r="E64" t="s">
+        <v>532</v>
+      </c>
+      <c r="F64" t="s">
+        <v>533</v>
+      </c>
+      <c r="G64" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="H64" t="s">
+        <v>246</v>
+      </c>
+      <c r="I64" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>42</v>
+      </c>
+      <c r="B65" t="s">
+        <v>408</v>
+      </c>
+      <c r="C65">
+        <v>980509994</v>
+      </c>
+      <c r="D65" t="s">
+        <v>406</v>
+      </c>
+      <c r="E65" t="s">
+        <v>534</v>
+      </c>
+      <c r="F65" t="s">
+        <v>535</v>
+      </c>
+      <c r="G65" s="1" t="s">
+        <v>407</v>
+      </c>
+      <c r="H65" t="s">
+        <v>257</v>
+      </c>
+      <c r="I65" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>43</v>
+      </c>
+      <c r="B66" t="s">
+        <v>232</v>
+      </c>
+      <c r="C66">
+        <v>925193206</v>
+      </c>
+      <c r="D66" t="s">
+        <v>233</v>
+      </c>
+      <c r="E66" t="s">
+        <v>536</v>
+      </c>
+      <c r="F66" t="s">
+        <v>537</v>
+      </c>
+      <c r="G66" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="H66" t="s">
+        <v>248</v>
+      </c>
+      <c r="I66" t="s">
+        <v>248</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{202A8526-E0EF-4475-93B0-7E089121C583}"/>
+    <hyperlink ref="D3" r:id="rId2" xr:uid="{4A53F7A7-E6A1-46DB-A0F3-1A937AF9E96F}"/>
+    <hyperlink ref="C4" r:id="rId3" display="tel:921619985" xr:uid="{74DB3D03-7F66-4ECA-BAF1-33C965146AD7}"/>
+    <hyperlink ref="D4" r:id="rId4" display="mailto:segovia@accem.es" xr:uid="{A83EA5F0-50D8-4869-B29C-CCA5AED8935C}"/>
+    <hyperlink ref="C5" r:id="rId5" display="tel:697163963(ext.:513)" xr:uid="{D5ECD482-4A67-4620-986A-DBA194FCBDB4}"/>
+    <hyperlink ref="D5" r:id="rId6" display="mailto:soria@accem.es" xr:uid="{39B0402A-2B53-4928-A696-27228F989459}"/>
+    <hyperlink ref="C6" r:id="rId7" display="tel:920256152" xr:uid="{8A12F64F-65C1-4C66-9A19-678A9559A44D}"/>
+    <hyperlink ref="C7" r:id="rId8" display="tel:947268620" xr:uid="{0D2EB532-F1B9-42B3-A526-F99F09C58849}"/>
+    <hyperlink ref="D7" r:id="rId9" display="mailto:burgos@accem.es" xr:uid="{2CB89887-0B50-4CF8-83F6-A6E47D635286}"/>
+    <hyperlink ref="C8" r:id="rId10" display="tel:987876143" xr:uid="{FA4CB35C-41EC-43CB-95EC-A94748FDC184}"/>
+    <hyperlink ref="D8" r:id="rId11" display="mailto:leon@accem.es" xr:uid="{3E5D042C-1280-4CFE-958E-AD3E6B2FC3F0}"/>
+    <hyperlink ref="D6" r:id="rId12" display="mailto:avila@accem.es" xr:uid="{FB78653A-1106-4B83-A278-830BBFEA75A6}"/>
+    <hyperlink ref="D11" r:id="rId13" xr:uid="{E3E9FA8E-A474-4A37-971C-5DD2A6FB0931}"/>
+    <hyperlink ref="D21" r:id="rId14" xr:uid="{FC00B382-8F42-492E-9738-28E12DFEA161}"/>
+    <hyperlink ref="D16" r:id="rId15" display="https://www.google.com/search?q=segovia%40cruzroja.es&amp;sca_esv=ba586742f70b6987&amp;rlz=1C1ONGR_esES1148ES1148&amp;biw=1920&amp;bih=911&amp;sxsrf=ANbL-n44hGuVhfV5QmGPOyCuypFS1rGLrA%3A1771606177476&amp;ei=oZCYaaTAHLXjkdUPg5380Ak&amp;ved=2ahUKEwjN6P6rw-iSAxVxRKQEHQCSK0cQgK4QegQIARAB&amp;uact=5&amp;oq=mail+cruz+roja+segovia&amp;gs_lp=Egxnd3Mtd2l6LXNlcnAiFm1haWwgY3J1eiByb2phIHNlZ292aWEyBRAhGKABMgUQIRifBTIFECEYnwUyBRAhGJ8FMgUQIRifBTIFECEYnwVItQlQvgNYpwhwAngBkAEAmAGmAaABoAeqAQMwLja4AQPIAQD4AQGYAgigAr0HwgIKEAAYsAMY1gQYR8ICBBAhGBWYAwCIBgGQBgiSBwMyLjagB9EgsgcDMC42uAe1B8IHBTAuNS4zyAcUgAgA&amp;sclient=gws-wiz-serp&amp;mstk=AUtExfC2HLYVd4A2ZkRLgXXtj06rHO-PzdbhzuKMDDil6wGKcs8xRtqfiMsb3XR_rW06WZv0PnEoofJQg5kyEVptPjAv5UP7LcKrdiR4golvKIznFin-CHa6w4MPx5hULFRlrFbhXQg_JdbdQneZVZXcLupU-sU_fuy26Sexdrj3nXUZFsrG2h-SFFnqnOcGtUEtAmQMhtPMAyF4sULxTRqa7Q2pPQ76HbxWqsE5usGgFht2nA&amp;csui=3" xr:uid="{ED51D852-5B9E-44D2-9A1D-BF35326327E3}"/>
+    <hyperlink ref="D17" r:id="rId16" display="https://www.google.com/search?q=burgos%40cruzroja.es&amp;sca_esv=ba586742f70b6987&amp;rlz=1C1ONGR_esES1148ES1148&amp;biw=1920&amp;bih=911&amp;sxsrf=ANbL-n4fZKsBH88TGCrNLOuMVuoZ5agKtA%3A1771606187423&amp;ei=q5CYaebGGfjw7M8P0J_gkA4&amp;ved=2ahUKEwjDm5Cww-iSAxWYQ6QEHSDHCKYQgK4QegQIARAC&amp;uact=5&amp;oq=mail+cruz+roja+burgos&amp;gs_lp=Egxnd3Mtd2l6LXNlcnAiFW1haWwgY3J1eiByb2phIGJ1cmdvczIFECEYoAEyBRAhGJ8FMgUQIRifBTIFECEYnwUyBRAhGJ8FMgUQIRifBTIFECEYnwUyBRAhGJ8FMgUQIRifBTIFECEYnwVInQpQzgVY7ghwAngBkAEAmAGpAaABywaqAQMwLja4AQPIAQD4AQGYAgigAuoGwgIKEAAYsAMY1gQYR8ICBBAhGBWYAwCIBgGQBgaSBwMyLjagB5MssgcDMC42uAfiBsIHBTAuNC40yAcVgAgA&amp;sclient=gws-wiz-serp&amp;mstk=AUtExfC-yucz8s9Cit2TK2UeuwXYQcp4sLkr5LQebDELtbjw2dLH825aqf6I5lcT9p7QQ0NZMlIrDuso_IC6Y1dmWTjtNQfsbMT4fx7-53Vz8lK70VlVqpzb-nNVHU14m0gV2LDerNCPmIEB2GIqRmQHzFPtZmk9ZPUxnahzwBURP0Nzr4H2zhJTa-TnjA_SB_M2ILAHncTyfbf2bD2v_jRaFROvO3Fd_XvZ-dZvu17tlKTAFg&amp;csui=3" xr:uid="{638BD4F7-B5C4-4FE4-803D-0B48C7FCB8CB}"/>
+    <hyperlink ref="D12" r:id="rId17" display="https://www.google.com/search?q=valladolid%40cruzroja.es&amp;sca_esv=ba586742f70b6987&amp;rlz=1C1ONGR_esES1148ES1148&amp;biw=1920&amp;bih=911&amp;sxsrf=ANbL-n65KhT7I-2k7iHIBCqcAKWOol7vpg%3A1771606207437&amp;ei=v5CYaay5GsGmkdUP6-ui8QE&amp;ved=2ahUKEwj_7ri5w-iSAxVQVKQEHd8bKYQQgK4QegQIARAC&amp;uact=5&amp;oq=mail+cruz+roja+valladolid&amp;gs_lp=Egxnd3Mtd2l6LXNlcnAiGW1haWwgY3J1eiByb2phIHZhbGxhZG9saWQyBRAhGJ8FMgUQIRifBTIFECEYnwUyBRAhGJ8FMgUQIRifBTIFECEYnwUyBRAhGJ8FMgUQIRifBTIFECEYnwUyBRAhGJ8FSL0MUI4DWP8KcAJ4AJABAJgBkwGgAcIJqgEEMC4xMLgBA8gBAPgBAZgCC6AC5AjCAgsQABiABBiwAxiiBMICCBAAGLADGO8FwgILEAAYsAMYogQYiQXCAgUQIRigAcICBBAhGBWYAwCIBgGQBgSSBwMyLjmgB-RSsgcDMC45uAffCMIHBTAuOC4zyAcdgAgA&amp;sclient=gws-wiz-serp&amp;mstk=AUtExfAMkrxKgxi2j9N0o2pWLYY53L3_GFeakmVJfK4TTXTzXesQUPACQdhohiMrhexBmUKcKO2RKiSz8lEC-RxirTQ8_uEerKfKggyq0eJEg_DCu9icVKEaCBZXvnAYRzjdylRpc7Tpb6UyEwLv0wgczVpN952ShDl2r-kJYizdkucuVnbeUOoPopmtDZejNfb_fYH-sWCXr4xwH8pFwubli63_P5WHXZPAvckTVXZHX4hQSQ&amp;csui=3" xr:uid="{FFBA2209-B28B-4766-9927-4230C3207778}"/>
+    <hyperlink ref="D13" r:id="rId18" display="https://www.google.com/search?q=valladolid%40cruzroja.es&amp;sca_esv=ba586742f70b6987&amp;rlz=1C1ONGR_esES1148ES1148&amp;biw=1920&amp;bih=911&amp;sxsrf=ANbL-n65KhT7I-2k7iHIBCqcAKWOol7vpg%3A1771606207437&amp;ei=v5CYaay5GsGmkdUP6-ui8QE&amp;ved=2ahUKEwj_7ri5w-iSAxVQVKQEHd8bKYQQgK4QegQIARAC&amp;uact=5&amp;oq=mail+cruz+roja+valladolid&amp;gs_lp=Egxnd3Mtd2l6LXNlcnAiGW1haWwgY3J1eiByb2phIHZhbGxhZG9saWQyBRAhGJ8FMgUQIRifBTIFECEYnwUyBRAhGJ8FMgUQIRifBTIFECEYnwUyBRAhGJ8FMgUQIRifBTIFECEYnwUyBRAhGJ8FSL0MUI4DWP8KcAJ4AJABAJgBkwGgAcIJqgEEMC4xMLgBA8gBAPgBAZgCC6AC5AjCAgsQABiABBiwAxiiBMICCBAAGLADGO8FwgILEAAYsAMYogQYiQXCAgUQIRigAcICBBAhGBWYAwCIBgGQBgSSBwMyLjmgB-RSsgcDMC45uAffCMIHBTAuOC4zyAcdgAgA&amp;sclient=gws-wiz-serp&amp;mstk=AUtExfAMkrxKgxi2j9N0o2pWLYY53L3_GFeakmVJfK4TTXTzXesQUPACQdhohiMrhexBmUKcKO2RKiSz8lEC-RxirTQ8_uEerKfKggyq0eJEg_DCu9icVKEaCBZXvnAYRzjdylRpc7Tpb6UyEwLv0wgczVpN952ShDl2r-kJYizdkucuVnbeUOoPopmtDZejNfb_fYH-sWCXr4xwH8pFwubli63_P5WHXZPAvckTVXZHX4hQSQ&amp;csui=3" xr:uid="{77F800E1-BD00-407B-A867-547D9EFD6B85}"/>
+    <hyperlink ref="D14" r:id="rId19" display="https://www.google.com/search?q=leon%40cruzroja.es&amp;sca_esv=ba586742f70b6987&amp;rlz=1C1ONGR_esES1148ES1148&amp;biw=1920&amp;bih=911&amp;sxsrf=ANbL-n45sJNoeKBVQNOzSdQe1vOuKExJrA%3A1771606215644&amp;ei=x5CYabSEJ8Ds7M8PitWQmQM&amp;ved=2ahUKEwirvOC-w-iSAxXJhP0HHapVFd4QgK4QegQIAhAC&amp;uact=5&amp;oq=mail+cruz+roja+le%C3%B3n&amp;gs_lp=Egxnd3Mtd2l6LXNlcnAiFG1haWwgY3J1eiByb2phIGxlw7NuMgUQIRigATIFECEYoAEyBRAhGJ8FMgUQIRifBTIFECEYnwUyBRAhGJ8FMgUQIRifBTIFECEYnwUyBRAhGJ8FMgUQIRifBUimC1DuBViuCXACeAGQAQCYAY4BoAH6A6oBAzAuNLgBA8gBAPgBAZgCBqACjwTCAgoQABiwAxjWBBhHwgIGEAAYFhgewgIIEAAYogQYiQXCAgUQABjvBcICBBAhGBWYAwCIBgGQBgiSBwMyLjSgB7AVsgcDMC40uAeIBMIHBTAuNC4yyAcOgAgA&amp;sclient=gws-wiz-serp&amp;mstk=AUtExfCgVbfRUcJ9wKiDfjVVbSJL20PUAWDE5kPVRwK3l8doRVtn7CGfosSxjlXivhqB7wc1ssOd7DeVwhNnL3GQHBwKC5eAlypVK6JxZVLW-AG1gsuiGYVwg8RlFPVwAsQhjI-l6rTvJb1-POIh1jXMBu3S7yi3vEkNLEcxmUyDmTJX7sJzNbEJ7jQI0LI4RdSw6froSRQsrkouNTRurqkc0aDBL9oac0HLoNCFlKhYIYmnNA&amp;csui=3" xr:uid="{D5B23C99-3319-4E27-AE1D-F33BDBF4152D}"/>
+    <hyperlink ref="D22" r:id="rId20" xr:uid="{9B8A9551-CECD-4049-8DAB-1033766D7897}"/>
+    <hyperlink ref="D23" r:id="rId21" xr:uid="{BDC308B1-F7CC-430A-9162-9B5EFD74313A}"/>
+    <hyperlink ref="D33" r:id="rId22" xr:uid="{6C94AE85-DB54-4391-9336-6144C0EFA778}"/>
+    <hyperlink ref="D34" r:id="rId23" xr:uid="{4940BAEB-55E6-423E-BD37-1CCA05DFA5A0}"/>
+    <hyperlink ref="D35" r:id="rId24" xr:uid="{9DA5C095-1547-4A8E-969F-A24BDF0ED14C}"/>
+    <hyperlink ref="D36" r:id="rId25" display="mailto:cd.caritasciudadrodrigo@caritas.es" xr:uid="{AD391B9B-B795-4690-AC9E-C316EFD57A02}"/>
+    <hyperlink ref="C38" r:id="rId26" display="tel:+34923219511" xr:uid="{218E4DD9-704B-4C57-A8FD-16836D59AD24}"/>
+    <hyperlink ref="D38" r:id="rId27" display="mailto:correo@casaescuelasantiagouno.es" xr:uid="{1242A272-66F1-4838-BA93-5FB2250715F0}"/>
+    <hyperlink ref="D39" r:id="rId28" xr:uid="{355258FE-4604-4126-AA49-C7CEB205BC36}"/>
+    <hyperlink ref="D40" r:id="rId29" xr:uid="{3B3B2471-6381-40D0-A7B3-EFFE1290CAF3}"/>
+    <hyperlink ref="D41" r:id="rId30" xr:uid="{DC1D1104-E629-4732-BC9B-A6C31675F28E}"/>
+    <hyperlink ref="D42" r:id="rId31" xr:uid="{CA924F34-3EDB-45DA-82B0-D70D4C28F127}"/>
+    <hyperlink ref="D43" r:id="rId32" xr:uid="{7B434DD4-887D-456E-8E14-20074CACF03C}"/>
+    <hyperlink ref="D44" r:id="rId33" display="mailto:caritas@caritasalamanca.org" xr:uid="{2FB9E28F-C288-4E63-B214-A479B2C0DD88}"/>
+    <hyperlink ref="D45" r:id="rId34" xr:uid="{8F9F7A21-179D-4313-AAE9-D8E4DE895340}"/>
+    <hyperlink ref="D46" r:id="rId35" xr:uid="{28B9782B-37CC-44C7-BACE-5B24ED823D6E}"/>
+    <hyperlink ref="D47" r:id="rId36" display="mailto:colectivo@cdrtcampos.es" xr:uid="{B6EC8623-6E1E-46DD-ADED-96E10539F53A}"/>
+    <hyperlink ref="D48" r:id="rId37" xr:uid="{CC8AA193-A71B-41AF-A45A-E5897FC4A958}"/>
+    <hyperlink ref="D50" r:id="rId38" xr:uid="{33668768-9D16-4A22-AE38-5CDAF71862C8}"/>
+    <hyperlink ref="D51" r:id="rId39" xr:uid="{61562734-741B-435F-9668-F332302D42E0}"/>
+    <hyperlink ref="D52" r:id="rId40" xr:uid="{7F91715B-6863-4CCB-AD9B-29DA143AC99F}"/>
+    <hyperlink ref="D53" r:id="rId41" xr:uid="{632D1B76-47C2-4025-B7A7-3421ABD4928B}"/>
+    <hyperlink ref="D54" r:id="rId42" xr:uid="{F9895957-C1D8-4260-8AC4-A8B096AF49F5}"/>
+    <hyperlink ref="D55" r:id="rId43" xr:uid="{EE2EB4E1-B964-4D87-A1B6-902365A88E80}"/>
+    <hyperlink ref="D56" r:id="rId44" display="mailto:diocesana@caritasvalladolid.es" xr:uid="{D98939C3-1EBF-47C1-8B60-9A9AB3974E4C}"/>
+    <hyperlink ref="C56" r:id="rId45" display="tel:983 20 23 01" xr:uid="{6FBCCCA8-C696-49A2-A81B-118F0D9427C7}"/>
+    <hyperlink ref="D57" r:id="rId46" xr:uid="{79B32847-0752-4D3C-93C0-0B4CFB97B2BE}"/>
+    <hyperlink ref="D58" r:id="rId47" xr:uid="{BF01541D-499C-400F-B53E-68D835B175A5}"/>
+    <hyperlink ref="C59" r:id="rId48" display="tel:983 62 05 30" xr:uid="{0A95C50C-88EB-42EB-AB5C-044374D60C48}"/>
+    <hyperlink ref="D59" r:id="rId49" xr:uid="{70F40A89-DDD4-4C38-99ED-17BBC32382A5}"/>
+    <hyperlink ref="D60" r:id="rId50" xr:uid="{B7503189-73BE-4BFF-8D19-917EDFE992E0}"/>
+    <hyperlink ref="D61" r:id="rId51" xr:uid="{0875480A-B399-4128-A0E5-EE6E7D0420C3}"/>
+    <hyperlink ref="D62" r:id="rId52" xr:uid="{4F343F3C-EB54-4068-9FA0-EAF3B13BCD75}"/>
+    <hyperlink ref="D63" r:id="rId53" xr:uid="{BB576755-B906-432F-A27D-8CC8448C194C}"/>
+    <hyperlink ref="D64" r:id="rId54" display="mailto:rosachacel@rosachacel.org" xr:uid="{BEAF3995-86F4-4E18-910A-E9363EC2931E}"/>
+    <hyperlink ref="D65" r:id="rId55" xr:uid="{45F01406-CFFA-4C08-B562-9D62E705D982}"/>
+    <hyperlink ref="D66" r:id="rId56" xr:uid="{06D24343-CEFB-481F-8B58-CBA86F72E2D4}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId57"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>